<commit_message>
Make multi-page quotes lay out correctly
Long estimates spilled onto a second page where the continued rows had
no column header and the totals block could end up stranded on its own,
because item rows auto-grew whenever a 工事品目 wrapped, so the page
break landed in an unpredictable place.

- fix the item row height and drop the body to 9pt, widen 工事品目 and
  trim 仕様/備考, so pagination is deterministic and ~17 lines fit a page
- repeat the table header row on every page and add a footer carrying the
  project name and "Page x / y"
- tighten the header block and the totals/remark block so a normal
  estimate still lands on a single sheet
- let the totals shrink to fit instead of rendering as ###

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/test_cyca_estimate_single_sheet_template.xlsx
+++ b/templates/test_cyca_estimate_single_sheet_template.xlsx
@@ -21,18 +21,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;¥&quot;#,##0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <b val="1"/>
-      <sz val="20"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -96,12 +91,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <b val="1"/>
-      <color rgb="001F3557"/>
-      <sz val="14"/>
     </font>
   </fonts>
   <fills count="4">
@@ -200,12 +189,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -214,70 +206,70 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -678,26 +670,26 @@
   <dimension ref="A2:H183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="4.5" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="6.5" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="11.5" customWidth="1" min="6" max="6"/>
+    <col width="14.5" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="10" customHeight="1"/>
-    <row r="2" ht="40" customHeight="1">
+    <row r="1" ht="6" customHeight="1"/>
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>御　見　積　書</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="26" customHeight="1">
+    <row r="3" ht="4" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1">
       <c r="A4" s="2" t="n"/>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -732,7 +724,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
+    <row r="10" ht="17" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>御 見 積 金 額</t>
@@ -740,7 +732,7 @@
       </c>
       <c r="C10" s="8" t="n"/>
     </row>
-    <row r="11" ht="20" customHeight="1"/>
+    <row r="11" ht="17" customHeight="1"/>
     <row r="12">
       <c r="C12" s="9" t="inlineStr">
         <is>
@@ -824,14 +816,14 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
           <t>工 事 内 容</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
+    <row r="21" ht="20" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
           <t>No.</t>
@@ -873,7 +865,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="27" customHeight="1">
       <c r="A22" s="16" t="n"/>
       <c r="B22" s="17" t="n"/>
       <c r="C22" s="17" t="n"/>
@@ -883,7 +875,7 @@
       <c r="G22" s="18" t="n"/>
       <c r="H22" s="17" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" ht="27" customHeight="1">
       <c r="A23" s="16" t="n"/>
       <c r="B23" s="17" t="n"/>
       <c r="C23" s="17" t="n"/>
@@ -893,7 +885,7 @@
       <c r="G23" s="18" t="n"/>
       <c r="H23" s="17" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="16" t="n"/>
       <c r="B24" s="17" t="n"/>
       <c r="C24" s="17" t="n"/>
@@ -903,7 +895,7 @@
       <c r="G24" s="18" t="n"/>
       <c r="H24" s="17" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="16" t="n"/>
       <c r="B25" s="17" t="n"/>
       <c r="C25" s="17" t="n"/>
@@ -913,7 +905,7 @@
       <c r="G25" s="18" t="n"/>
       <c r="H25" s="17" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="16" t="n"/>
       <c r="B26" s="17" t="n"/>
       <c r="C26" s="17" t="n"/>
@@ -923,7 +915,7 @@
       <c r="G26" s="18" t="n"/>
       <c r="H26" s="17" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="16" t="n"/>
       <c r="B27" s="17" t="n"/>
       <c r="C27" s="17" t="n"/>
@@ -933,7 +925,7 @@
       <c r="G27" s="18" t="n"/>
       <c r="H27" s="17" t="n"/>
     </row>
-    <row r="28">
+    <row r="28" ht="27" customHeight="1">
       <c r="A28" s="16" t="n"/>
       <c r="B28" s="17" t="n"/>
       <c r="C28" s="17" t="n"/>
@@ -943,7 +935,7 @@
       <c r="G28" s="18" t="n"/>
       <c r="H28" s="17" t="n"/>
     </row>
-    <row r="29">
+    <row r="29" ht="27" customHeight="1">
       <c r="A29" s="16" t="n"/>
       <c r="B29" s="17" t="n"/>
       <c r="C29" s="17" t="n"/>
@@ -953,7 +945,7 @@
       <c r="G29" s="18" t="n"/>
       <c r="H29" s="17" t="n"/>
     </row>
-    <row r="30">
+    <row r="30" ht="27" customHeight="1">
       <c r="A30" s="16" t="n"/>
       <c r="B30" s="17" t="n"/>
       <c r="C30" s="17" t="n"/>
@@ -963,7 +955,7 @@
       <c r="G30" s="18" t="n"/>
       <c r="H30" s="17" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" ht="27" customHeight="1">
       <c r="A31" s="16" t="n"/>
       <c r="B31" s="17" t="n"/>
       <c r="C31" s="17" t="n"/>
@@ -973,7 +965,7 @@
       <c r="G31" s="18" t="n"/>
       <c r="H31" s="17" t="n"/>
     </row>
-    <row r="32">
+    <row r="32" ht="27" customHeight="1">
       <c r="A32" s="16" t="n"/>
       <c r="B32" s="17" t="n"/>
       <c r="C32" s="17" t="n"/>
@@ -983,7 +975,7 @@
       <c r="G32" s="18" t="n"/>
       <c r="H32" s="17" t="n"/>
     </row>
-    <row r="33">
+    <row r="33" ht="27" customHeight="1">
       <c r="A33" s="16" t="n"/>
       <c r="B33" s="17" t="n"/>
       <c r="C33" s="17" t="n"/>
@@ -993,7 +985,7 @@
       <c r="G33" s="18" t="n"/>
       <c r="H33" s="17" t="n"/>
     </row>
-    <row r="34">
+    <row r="34" ht="27" customHeight="1">
       <c r="A34" s="16" t="n"/>
       <c r="B34" s="17" t="n"/>
       <c r="C34" s="17" t="n"/>
@@ -1003,7 +995,7 @@
       <c r="G34" s="18" t="n"/>
       <c r="H34" s="17" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" ht="27" customHeight="1">
       <c r="A35" s="16" t="n"/>
       <c r="B35" s="17" t="n"/>
       <c r="C35" s="17" t="n"/>
@@ -1013,7 +1005,7 @@
       <c r="G35" s="18" t="n"/>
       <c r="H35" s="17" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="27" customHeight="1">
       <c r="A36" s="16" t="n"/>
       <c r="B36" s="17" t="n"/>
       <c r="C36" s="17" t="n"/>
@@ -1023,7 +1015,7 @@
       <c r="G36" s="18" t="n"/>
       <c r="H36" s="17" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" ht="27" customHeight="1">
       <c r="A37" s="16" t="n"/>
       <c r="B37" s="17" t="n"/>
       <c r="C37" s="17" t="n"/>
@@ -1033,7 +1025,7 @@
       <c r="G37" s="18" t="n"/>
       <c r="H37" s="17" t="n"/>
     </row>
-    <row r="38">
+    <row r="38" ht="27" customHeight="1">
       <c r="A38" s="16" t="n"/>
       <c r="B38" s="17" t="n"/>
       <c r="C38" s="17" t="n"/>
@@ -1043,7 +1035,7 @@
       <c r="G38" s="18" t="n"/>
       <c r="H38" s="17" t="n"/>
     </row>
-    <row r="39">
+    <row r="39" ht="27" customHeight="1">
       <c r="A39" s="16" t="n"/>
       <c r="B39" s="17" t="n"/>
       <c r="C39" s="17" t="n"/>
@@ -1053,7 +1045,7 @@
       <c r="G39" s="18" t="n"/>
       <c r="H39" s="17" t="n"/>
     </row>
-    <row r="40">
+    <row r="40" ht="27" customHeight="1">
       <c r="A40" s="16" t="n"/>
       <c r="B40" s="17" t="n"/>
       <c r="C40" s="17" t="n"/>
@@ -1063,7 +1055,7 @@
       <c r="G40" s="18" t="n"/>
       <c r="H40" s="17" t="n"/>
     </row>
-    <row r="41">
+    <row r="41" ht="27" customHeight="1">
       <c r="A41" s="16" t="n"/>
       <c r="B41" s="17" t="n"/>
       <c r="C41" s="17" t="n"/>
@@ -1073,7 +1065,7 @@
       <c r="G41" s="18" t="n"/>
       <c r="H41" s="17" t="n"/>
     </row>
-    <row r="42">
+    <row r="42" ht="27" customHeight="1">
       <c r="A42" s="16" t="n"/>
       <c r="B42" s="17" t="n"/>
       <c r="C42" s="17" t="n"/>
@@ -1083,7 +1075,7 @@
       <c r="G42" s="18" t="n"/>
       <c r="H42" s="17" t="n"/>
     </row>
-    <row r="43">
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="16" t="n"/>
       <c r="B43" s="17" t="n"/>
       <c r="C43" s="17" t="n"/>
@@ -1093,7 +1085,7 @@
       <c r="G43" s="18" t="n"/>
       <c r="H43" s="17" t="n"/>
     </row>
-    <row r="44">
+    <row r="44" ht="27" customHeight="1">
       <c r="A44" s="16" t="n"/>
       <c r="B44" s="17" t="n"/>
       <c r="C44" s="17" t="n"/>
@@ -1103,7 +1095,7 @@
       <c r="G44" s="18" t="n"/>
       <c r="H44" s="17" t="n"/>
     </row>
-    <row r="45">
+    <row r="45" ht="27" customHeight="1">
       <c r="A45" s="16" t="n"/>
       <c r="B45" s="17" t="n"/>
       <c r="C45" s="17" t="n"/>
@@ -1113,7 +1105,7 @@
       <c r="G45" s="18" t="n"/>
       <c r="H45" s="17" t="n"/>
     </row>
-    <row r="46">
+    <row r="46" ht="27" customHeight="1">
       <c r="A46" s="16" t="n"/>
       <c r="B46" s="17" t="n"/>
       <c r="C46" s="17" t="n"/>
@@ -1123,7 +1115,7 @@
       <c r="G46" s="18" t="n"/>
       <c r="H46" s="17" t="n"/>
     </row>
-    <row r="47">
+    <row r="47" ht="27" customHeight="1">
       <c r="A47" s="16" t="n"/>
       <c r="B47" s="17" t="n"/>
       <c r="C47" s="17" t="n"/>
@@ -1133,7 +1125,7 @@
       <c r="G47" s="18" t="n"/>
       <c r="H47" s="17" t="n"/>
     </row>
-    <row r="48">
+    <row r="48" ht="27" customHeight="1">
       <c r="A48" s="16" t="n"/>
       <c r="B48" s="17" t="n"/>
       <c r="C48" s="17" t="n"/>
@@ -1143,7 +1135,7 @@
       <c r="G48" s="18" t="n"/>
       <c r="H48" s="17" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" ht="27" customHeight="1">
       <c r="A49" s="16" t="n"/>
       <c r="B49" s="17" t="n"/>
       <c r="C49" s="17" t="n"/>
@@ -1153,7 +1145,7 @@
       <c r="G49" s="18" t="n"/>
       <c r="H49" s="17" t="n"/>
     </row>
-    <row r="50">
+    <row r="50" ht="27" customHeight="1">
       <c r="A50" s="16" t="n"/>
       <c r="B50" s="17" t="n"/>
       <c r="C50" s="17" t="n"/>
@@ -1163,7 +1155,7 @@
       <c r="G50" s="18" t="n"/>
       <c r="H50" s="17" t="n"/>
     </row>
-    <row r="51">
+    <row r="51" ht="27" customHeight="1">
       <c r="A51" s="16" t="n"/>
       <c r="B51" s="17" t="n"/>
       <c r="C51" s="17" t="n"/>
@@ -1173,7 +1165,7 @@
       <c r="G51" s="18" t="n"/>
       <c r="H51" s="17" t="n"/>
     </row>
-    <row r="52">
+    <row r="52" ht="27" customHeight="1">
       <c r="A52" s="16" t="n"/>
       <c r="B52" s="17" t="n"/>
       <c r="C52" s="17" t="n"/>
@@ -1183,7 +1175,7 @@
       <c r="G52" s="18" t="n"/>
       <c r="H52" s="17" t="n"/>
     </row>
-    <row r="53">
+    <row r="53" ht="27" customHeight="1">
       <c r="A53" s="16" t="n"/>
       <c r="B53" s="17" t="n"/>
       <c r="C53" s="17" t="n"/>
@@ -1193,7 +1185,7 @@
       <c r="G53" s="18" t="n"/>
       <c r="H53" s="17" t="n"/>
     </row>
-    <row r="54">
+    <row r="54" ht="27" customHeight="1">
       <c r="A54" s="16" t="n"/>
       <c r="B54" s="17" t="n"/>
       <c r="C54" s="17" t="n"/>
@@ -1203,7 +1195,7 @@
       <c r="G54" s="18" t="n"/>
       <c r="H54" s="17" t="n"/>
     </row>
-    <row r="55">
+    <row r="55" ht="27" customHeight="1">
       <c r="A55" s="16" t="n"/>
       <c r="B55" s="17" t="n"/>
       <c r="C55" s="17" t="n"/>
@@ -1213,7 +1205,7 @@
       <c r="G55" s="18" t="n"/>
       <c r="H55" s="17" t="n"/>
     </row>
-    <row r="56">
+    <row r="56" ht="27" customHeight="1">
       <c r="A56" s="16" t="n"/>
       <c r="B56" s="17" t="n"/>
       <c r="C56" s="17" t="n"/>
@@ -1223,7 +1215,7 @@
       <c r="G56" s="18" t="n"/>
       <c r="H56" s="17" t="n"/>
     </row>
-    <row r="57">
+    <row r="57" ht="27" customHeight="1">
       <c r="A57" s="16" t="n"/>
       <c r="B57" s="17" t="n"/>
       <c r="C57" s="17" t="n"/>
@@ -1233,7 +1225,7 @@
       <c r="G57" s="18" t="n"/>
       <c r="H57" s="17" t="n"/>
     </row>
-    <row r="58">
+    <row r="58" ht="27" customHeight="1">
       <c r="A58" s="16" t="n"/>
       <c r="B58" s="17" t="n"/>
       <c r="C58" s="17" t="n"/>
@@ -1243,7 +1235,7 @@
       <c r="G58" s="18" t="n"/>
       <c r="H58" s="17" t="n"/>
     </row>
-    <row r="59">
+    <row r="59" ht="27" customHeight="1">
       <c r="A59" s="16" t="n"/>
       <c r="B59" s="17" t="n"/>
       <c r="C59" s="17" t="n"/>
@@ -1253,7 +1245,7 @@
       <c r="G59" s="18" t="n"/>
       <c r="H59" s="17" t="n"/>
     </row>
-    <row r="60">
+    <row r="60" ht="27" customHeight="1">
       <c r="A60" s="16" t="n"/>
       <c r="B60" s="17" t="n"/>
       <c r="C60" s="17" t="n"/>
@@ -1263,7 +1255,7 @@
       <c r="G60" s="18" t="n"/>
       <c r="H60" s="17" t="n"/>
     </row>
-    <row r="61">
+    <row r="61" ht="27" customHeight="1">
       <c r="A61" s="16" t="n"/>
       <c r="B61" s="17" t="n"/>
       <c r="C61" s="17" t="n"/>
@@ -1273,7 +1265,7 @@
       <c r="G61" s="18" t="n"/>
       <c r="H61" s="17" t="n"/>
     </row>
-    <row r="62">
+    <row r="62" ht="27" customHeight="1">
       <c r="A62" s="16" t="n"/>
       <c r="B62" s="17" t="n"/>
       <c r="C62" s="17" t="n"/>
@@ -1283,7 +1275,7 @@
       <c r="G62" s="18" t="n"/>
       <c r="H62" s="17" t="n"/>
     </row>
-    <row r="63">
+    <row r="63" ht="27" customHeight="1">
       <c r="A63" s="16" t="n"/>
       <c r="B63" s="17" t="n"/>
       <c r="C63" s="17" t="n"/>
@@ -1293,7 +1285,7 @@
       <c r="G63" s="18" t="n"/>
       <c r="H63" s="17" t="n"/>
     </row>
-    <row r="64">
+    <row r="64" ht="27" customHeight="1">
       <c r="A64" s="16" t="n"/>
       <c r="B64" s="17" t="n"/>
       <c r="C64" s="17" t="n"/>
@@ -1303,7 +1295,7 @@
       <c r="G64" s="18" t="n"/>
       <c r="H64" s="17" t="n"/>
     </row>
-    <row r="65">
+    <row r="65" ht="27" customHeight="1">
       <c r="A65" s="16" t="n"/>
       <c r="B65" s="17" t="n"/>
       <c r="C65" s="17" t="n"/>
@@ -1313,7 +1305,7 @@
       <c r="G65" s="18" t="n"/>
       <c r="H65" s="17" t="n"/>
     </row>
-    <row r="66">
+    <row r="66" ht="27" customHeight="1">
       <c r="A66" s="16" t="n"/>
       <c r="B66" s="17" t="n"/>
       <c r="C66" s="17" t="n"/>
@@ -1323,7 +1315,7 @@
       <c r="G66" s="18" t="n"/>
       <c r="H66" s="17" t="n"/>
     </row>
-    <row r="67">
+    <row r="67" ht="27" customHeight="1">
       <c r="A67" s="16" t="n"/>
       <c r="B67" s="17" t="n"/>
       <c r="C67" s="17" t="n"/>
@@ -1333,7 +1325,7 @@
       <c r="G67" s="18" t="n"/>
       <c r="H67" s="17" t="n"/>
     </row>
-    <row r="68">
+    <row r="68" ht="27" customHeight="1">
       <c r="A68" s="16" t="n"/>
       <c r="B68" s="17" t="n"/>
       <c r="C68" s="17" t="n"/>
@@ -1343,7 +1335,7 @@
       <c r="G68" s="18" t="n"/>
       <c r="H68" s="17" t="n"/>
     </row>
-    <row r="69">
+    <row r="69" ht="27" customHeight="1">
       <c r="A69" s="16" t="n"/>
       <c r="B69" s="17" t="n"/>
       <c r="C69" s="17" t="n"/>
@@ -1353,7 +1345,7 @@
       <c r="G69" s="18" t="n"/>
       <c r="H69" s="17" t="n"/>
     </row>
-    <row r="70">
+    <row r="70" ht="27" customHeight="1">
       <c r="A70" s="16" t="n"/>
       <c r="B70" s="17" t="n"/>
       <c r="C70" s="17" t="n"/>
@@ -1363,7 +1355,7 @@
       <c r="G70" s="18" t="n"/>
       <c r="H70" s="17" t="n"/>
     </row>
-    <row r="71">
+    <row r="71" ht="27" customHeight="1">
       <c r="A71" s="16" t="n"/>
       <c r="B71" s="17" t="n"/>
       <c r="C71" s="17" t="n"/>
@@ -1373,7 +1365,7 @@
       <c r="G71" s="18" t="n"/>
       <c r="H71" s="17" t="n"/>
     </row>
-    <row r="72">
+    <row r="72" ht="27" customHeight="1">
       <c r="A72" s="16" t="n"/>
       <c r="B72" s="17" t="n"/>
       <c r="C72" s="17" t="n"/>
@@ -1383,7 +1375,7 @@
       <c r="G72" s="18" t="n"/>
       <c r="H72" s="17" t="n"/>
     </row>
-    <row r="73">
+    <row r="73" ht="27" customHeight="1">
       <c r="A73" s="16" t="n"/>
       <c r="B73" s="17" t="n"/>
       <c r="C73" s="17" t="n"/>
@@ -1393,7 +1385,7 @@
       <c r="G73" s="18" t="n"/>
       <c r="H73" s="17" t="n"/>
     </row>
-    <row r="74">
+    <row r="74" ht="27" customHeight="1">
       <c r="A74" s="16" t="n"/>
       <c r="B74" s="17" t="n"/>
       <c r="C74" s="17" t="n"/>
@@ -1403,7 +1395,7 @@
       <c r="G74" s="18" t="n"/>
       <c r="H74" s="17" t="n"/>
     </row>
-    <row r="75">
+    <row r="75" ht="27" customHeight="1">
       <c r="A75" s="16" t="n"/>
       <c r="B75" s="17" t="n"/>
       <c r="C75" s="17" t="n"/>
@@ -1413,7 +1405,7 @@
       <c r="G75" s="18" t="n"/>
       <c r="H75" s="17" t="n"/>
     </row>
-    <row r="76">
+    <row r="76" ht="27" customHeight="1">
       <c r="A76" s="16" t="n"/>
       <c r="B76" s="17" t="n"/>
       <c r="C76" s="17" t="n"/>
@@ -1423,7 +1415,7 @@
       <c r="G76" s="18" t="n"/>
       <c r="H76" s="17" t="n"/>
     </row>
-    <row r="77">
+    <row r="77" ht="27" customHeight="1">
       <c r="A77" s="16" t="n"/>
       <c r="B77" s="17" t="n"/>
       <c r="C77" s="17" t="n"/>
@@ -1433,7 +1425,7 @@
       <c r="G77" s="18" t="n"/>
       <c r="H77" s="17" t="n"/>
     </row>
-    <row r="78">
+    <row r="78" ht="27" customHeight="1">
       <c r="A78" s="16" t="n"/>
       <c r="B78" s="17" t="n"/>
       <c r="C78" s="17" t="n"/>
@@ -1443,7 +1435,7 @@
       <c r="G78" s="18" t="n"/>
       <c r="H78" s="17" t="n"/>
     </row>
-    <row r="79">
+    <row r="79" ht="27" customHeight="1">
       <c r="A79" s="16" t="n"/>
       <c r="B79" s="17" t="n"/>
       <c r="C79" s="17" t="n"/>
@@ -1453,7 +1445,7 @@
       <c r="G79" s="18" t="n"/>
       <c r="H79" s="17" t="n"/>
     </row>
-    <row r="80">
+    <row r="80" ht="27" customHeight="1">
       <c r="A80" s="16" t="n"/>
       <c r="B80" s="17" t="n"/>
       <c r="C80" s="17" t="n"/>
@@ -1463,7 +1455,7 @@
       <c r="G80" s="18" t="n"/>
       <c r="H80" s="17" t="n"/>
     </row>
-    <row r="81">
+    <row r="81" ht="27" customHeight="1">
       <c r="A81" s="16" t="n"/>
       <c r="B81" s="17" t="n"/>
       <c r="C81" s="17" t="n"/>
@@ -1473,7 +1465,7 @@
       <c r="G81" s="18" t="n"/>
       <c r="H81" s="17" t="n"/>
     </row>
-    <row r="82">
+    <row r="82" ht="27" customHeight="1">
       <c r="A82" s="16" t="n"/>
       <c r="B82" s="17" t="n"/>
       <c r="C82" s="17" t="n"/>
@@ -1483,7 +1475,7 @@
       <c r="G82" s="18" t="n"/>
       <c r="H82" s="17" t="n"/>
     </row>
-    <row r="83">
+    <row r="83" ht="27" customHeight="1">
       <c r="A83" s="16" t="n"/>
       <c r="B83" s="17" t="n"/>
       <c r="C83" s="17" t="n"/>
@@ -1493,7 +1485,7 @@
       <c r="G83" s="18" t="n"/>
       <c r="H83" s="17" t="n"/>
     </row>
-    <row r="84">
+    <row r="84" ht="27" customHeight="1">
       <c r="A84" s="16" t="n"/>
       <c r="B84" s="17" t="n"/>
       <c r="C84" s="17" t="n"/>
@@ -1503,7 +1495,7 @@
       <c r="G84" s="18" t="n"/>
       <c r="H84" s="17" t="n"/>
     </row>
-    <row r="85">
+    <row r="85" ht="27" customHeight="1">
       <c r="A85" s="16" t="n"/>
       <c r="B85" s="17" t="n"/>
       <c r="C85" s="17" t="n"/>
@@ -1513,7 +1505,7 @@
       <c r="G85" s="18" t="n"/>
       <c r="H85" s="17" t="n"/>
     </row>
-    <row r="86">
+    <row r="86" ht="27" customHeight="1">
       <c r="A86" s="16" t="n"/>
       <c r="B86" s="17" t="n"/>
       <c r="C86" s="17" t="n"/>
@@ -1523,7 +1515,7 @@
       <c r="G86" s="18" t="n"/>
       <c r="H86" s="17" t="n"/>
     </row>
-    <row r="87">
+    <row r="87" ht="27" customHeight="1">
       <c r="A87" s="16" t="n"/>
       <c r="B87" s="17" t="n"/>
       <c r="C87" s="17" t="n"/>
@@ -1533,7 +1525,7 @@
       <c r="G87" s="18" t="n"/>
       <c r="H87" s="17" t="n"/>
     </row>
-    <row r="88">
+    <row r="88" ht="27" customHeight="1">
       <c r="A88" s="16" t="n"/>
       <c r="B88" s="17" t="n"/>
       <c r="C88" s="17" t="n"/>
@@ -1543,7 +1535,7 @@
       <c r="G88" s="18" t="n"/>
       <c r="H88" s="17" t="n"/>
     </row>
-    <row r="89">
+    <row r="89" ht="27" customHeight="1">
       <c r="A89" s="16" t="n"/>
       <c r="B89" s="17" t="n"/>
       <c r="C89" s="17" t="n"/>
@@ -1553,7 +1545,7 @@
       <c r="G89" s="18" t="n"/>
       <c r="H89" s="17" t="n"/>
     </row>
-    <row r="90">
+    <row r="90" ht="27" customHeight="1">
       <c r="A90" s="16" t="n"/>
       <c r="B90" s="17" t="n"/>
       <c r="C90" s="17" t="n"/>
@@ -1563,7 +1555,7 @@
       <c r="G90" s="18" t="n"/>
       <c r="H90" s="17" t="n"/>
     </row>
-    <row r="91">
+    <row r="91" ht="27" customHeight="1">
       <c r="A91" s="16" t="n"/>
       <c r="B91" s="17" t="n"/>
       <c r="C91" s="17" t="n"/>
@@ -1573,7 +1565,7 @@
       <c r="G91" s="18" t="n"/>
       <c r="H91" s="17" t="n"/>
     </row>
-    <row r="92">
+    <row r="92" ht="27" customHeight="1">
       <c r="A92" s="16" t="n"/>
       <c r="B92" s="17" t="n"/>
       <c r="C92" s="17" t="n"/>
@@ -1583,7 +1575,7 @@
       <c r="G92" s="18" t="n"/>
       <c r="H92" s="17" t="n"/>
     </row>
-    <row r="93">
+    <row r="93" ht="27" customHeight="1">
       <c r="A93" s="16" t="n"/>
       <c r="B93" s="17" t="n"/>
       <c r="C93" s="17" t="n"/>
@@ -1593,7 +1585,7 @@
       <c r="G93" s="18" t="n"/>
       <c r="H93" s="17" t="n"/>
     </row>
-    <row r="94">
+    <row r="94" ht="27" customHeight="1">
       <c r="A94" s="16" t="n"/>
       <c r="B94" s="17" t="n"/>
       <c r="C94" s="17" t="n"/>
@@ -1603,7 +1595,7 @@
       <c r="G94" s="18" t="n"/>
       <c r="H94" s="17" t="n"/>
     </row>
-    <row r="95">
+    <row r="95" ht="27" customHeight="1">
       <c r="A95" s="16" t="n"/>
       <c r="B95" s="17" t="n"/>
       <c r="C95" s="17" t="n"/>
@@ -1613,7 +1605,7 @@
       <c r="G95" s="18" t="n"/>
       <c r="H95" s="17" t="n"/>
     </row>
-    <row r="96">
+    <row r="96" ht="27" customHeight="1">
       <c r="A96" s="16" t="n"/>
       <c r="B96" s="17" t="n"/>
       <c r="C96" s="17" t="n"/>
@@ -1623,7 +1615,7 @@
       <c r="G96" s="18" t="n"/>
       <c r="H96" s="17" t="n"/>
     </row>
-    <row r="97">
+    <row r="97" ht="27" customHeight="1">
       <c r="A97" s="16" t="n"/>
       <c r="B97" s="17" t="n"/>
       <c r="C97" s="17" t="n"/>
@@ -1633,7 +1625,7 @@
       <c r="G97" s="18" t="n"/>
       <c r="H97" s="17" t="n"/>
     </row>
-    <row r="98">
+    <row r="98" ht="27" customHeight="1">
       <c r="A98" s="16" t="n"/>
       <c r="B98" s="17" t="n"/>
       <c r="C98" s="17" t="n"/>
@@ -1643,7 +1635,7 @@
       <c r="G98" s="18" t="n"/>
       <c r="H98" s="17" t="n"/>
     </row>
-    <row r="99">
+    <row r="99" ht="27" customHeight="1">
       <c r="A99" s="16" t="n"/>
       <c r="B99" s="17" t="n"/>
       <c r="C99" s="17" t="n"/>
@@ -1653,7 +1645,7 @@
       <c r="G99" s="18" t="n"/>
       <c r="H99" s="17" t="n"/>
     </row>
-    <row r="100">
+    <row r="100" ht="27" customHeight="1">
       <c r="A100" s="16" t="n"/>
       <c r="B100" s="17" t="n"/>
       <c r="C100" s="17" t="n"/>
@@ -1663,7 +1655,7 @@
       <c r="G100" s="18" t="n"/>
       <c r="H100" s="17" t="n"/>
     </row>
-    <row r="101">
+    <row r="101" ht="27" customHeight="1">
       <c r="A101" s="16" t="n"/>
       <c r="B101" s="17" t="n"/>
       <c r="C101" s="17" t="n"/>
@@ -1673,7 +1665,7 @@
       <c r="G101" s="18" t="n"/>
       <c r="H101" s="17" t="n"/>
     </row>
-    <row r="102">
+    <row r="102" ht="27" customHeight="1">
       <c r="A102" s="16" t="n"/>
       <c r="B102" s="17" t="n"/>
       <c r="C102" s="17" t="n"/>
@@ -1683,7 +1675,7 @@
       <c r="G102" s="18" t="n"/>
       <c r="H102" s="17" t="n"/>
     </row>
-    <row r="103">
+    <row r="103" ht="27" customHeight="1">
       <c r="A103" s="16" t="n"/>
       <c r="B103" s="17" t="n"/>
       <c r="C103" s="17" t="n"/>
@@ -1693,7 +1685,7 @@
       <c r="G103" s="18" t="n"/>
       <c r="H103" s="17" t="n"/>
     </row>
-    <row r="104">
+    <row r="104" ht="27" customHeight="1">
       <c r="A104" s="16" t="n"/>
       <c r="B104" s="17" t="n"/>
       <c r="C104" s="17" t="n"/>
@@ -1703,7 +1695,7 @@
       <c r="G104" s="18" t="n"/>
       <c r="H104" s="17" t="n"/>
     </row>
-    <row r="105">
+    <row r="105" ht="27" customHeight="1">
       <c r="A105" s="16" t="n"/>
       <c r="B105" s="17" t="n"/>
       <c r="C105" s="17" t="n"/>
@@ -1713,7 +1705,7 @@
       <c r="G105" s="18" t="n"/>
       <c r="H105" s="17" t="n"/>
     </row>
-    <row r="106">
+    <row r="106" ht="27" customHeight="1">
       <c r="A106" s="16" t="n"/>
       <c r="B106" s="17" t="n"/>
       <c r="C106" s="17" t="n"/>
@@ -1723,7 +1715,7 @@
       <c r="G106" s="18" t="n"/>
       <c r="H106" s="17" t="n"/>
     </row>
-    <row r="107">
+    <row r="107" ht="27" customHeight="1">
       <c r="A107" s="16" t="n"/>
       <c r="B107" s="17" t="n"/>
       <c r="C107" s="17" t="n"/>
@@ -1733,7 +1725,7 @@
       <c r="G107" s="18" t="n"/>
       <c r="H107" s="17" t="n"/>
     </row>
-    <row r="108">
+    <row r="108" ht="27" customHeight="1">
       <c r="A108" s="16" t="n"/>
       <c r="B108" s="17" t="n"/>
       <c r="C108" s="17" t="n"/>
@@ -1743,7 +1735,7 @@
       <c r="G108" s="18" t="n"/>
       <c r="H108" s="17" t="n"/>
     </row>
-    <row r="109">
+    <row r="109" ht="27" customHeight="1">
       <c r="A109" s="16" t="n"/>
       <c r="B109" s="17" t="n"/>
       <c r="C109" s="17" t="n"/>
@@ -1753,7 +1745,7 @@
       <c r="G109" s="18" t="n"/>
       <c r="H109" s="17" t="n"/>
     </row>
-    <row r="110">
+    <row r="110" ht="27" customHeight="1">
       <c r="A110" s="16" t="n"/>
       <c r="B110" s="17" t="n"/>
       <c r="C110" s="17" t="n"/>
@@ -1763,7 +1755,7 @@
       <c r="G110" s="18" t="n"/>
       <c r="H110" s="17" t="n"/>
     </row>
-    <row r="111">
+    <row r="111" ht="27" customHeight="1">
       <c r="A111" s="16" t="n"/>
       <c r="B111" s="17" t="n"/>
       <c r="C111" s="17" t="n"/>
@@ -1773,7 +1765,7 @@
       <c r="G111" s="18" t="n"/>
       <c r="H111" s="17" t="n"/>
     </row>
-    <row r="112">
+    <row r="112" ht="27" customHeight="1">
       <c r="A112" s="16" t="n"/>
       <c r="B112" s="17" t="n"/>
       <c r="C112" s="17" t="n"/>
@@ -1783,7 +1775,7 @@
       <c r="G112" s="18" t="n"/>
       <c r="H112" s="17" t="n"/>
     </row>
-    <row r="113">
+    <row r="113" ht="27" customHeight="1">
       <c r="A113" s="16" t="n"/>
       <c r="B113" s="17" t="n"/>
       <c r="C113" s="17" t="n"/>
@@ -1793,7 +1785,7 @@
       <c r="G113" s="18" t="n"/>
       <c r="H113" s="17" t="n"/>
     </row>
-    <row r="114">
+    <row r="114" ht="27" customHeight="1">
       <c r="A114" s="16" t="n"/>
       <c r="B114" s="17" t="n"/>
       <c r="C114" s="17" t="n"/>
@@ -1803,7 +1795,7 @@
       <c r="G114" s="18" t="n"/>
       <c r="H114" s="17" t="n"/>
     </row>
-    <row r="115">
+    <row r="115" ht="27" customHeight="1">
       <c r="A115" s="16" t="n"/>
       <c r="B115" s="17" t="n"/>
       <c r="C115" s="17" t="n"/>
@@ -1813,7 +1805,7 @@
       <c r="G115" s="18" t="n"/>
       <c r="H115" s="17" t="n"/>
     </row>
-    <row r="116">
+    <row r="116" ht="27" customHeight="1">
       <c r="A116" s="16" t="n"/>
       <c r="B116" s="17" t="n"/>
       <c r="C116" s="17" t="n"/>
@@ -1823,7 +1815,7 @@
       <c r="G116" s="18" t="n"/>
       <c r="H116" s="17" t="n"/>
     </row>
-    <row r="117">
+    <row r="117" ht="27" customHeight="1">
       <c r="A117" s="16" t="n"/>
       <c r="B117" s="17" t="n"/>
       <c r="C117" s="17" t="n"/>
@@ -1833,7 +1825,7 @@
       <c r="G117" s="18" t="n"/>
       <c r="H117" s="17" t="n"/>
     </row>
-    <row r="118">
+    <row r="118" ht="27" customHeight="1">
       <c r="A118" s="16" t="n"/>
       <c r="B118" s="17" t="n"/>
       <c r="C118" s="17" t="n"/>
@@ -1843,7 +1835,7 @@
       <c r="G118" s="18" t="n"/>
       <c r="H118" s="17" t="n"/>
     </row>
-    <row r="119">
+    <row r="119" ht="27" customHeight="1">
       <c r="A119" s="16" t="n"/>
       <c r="B119" s="17" t="n"/>
       <c r="C119" s="17" t="n"/>
@@ -1853,7 +1845,7 @@
       <c r="G119" s="18" t="n"/>
       <c r="H119" s="17" t="n"/>
     </row>
-    <row r="120">
+    <row r="120" ht="27" customHeight="1">
       <c r="A120" s="16" t="n"/>
       <c r="B120" s="17" t="n"/>
       <c r="C120" s="17" t="n"/>
@@ -1863,7 +1855,7 @@
       <c r="G120" s="18" t="n"/>
       <c r="H120" s="17" t="n"/>
     </row>
-    <row r="121">
+    <row r="121" ht="27" customHeight="1">
       <c r="A121" s="16" t="n"/>
       <c r="B121" s="17" t="n"/>
       <c r="C121" s="17" t="n"/>
@@ -1873,7 +1865,7 @@
       <c r="G121" s="18" t="n"/>
       <c r="H121" s="17" t="n"/>
     </row>
-    <row r="122">
+    <row r="122" ht="27" customHeight="1">
       <c r="A122" s="16" t="n"/>
       <c r="B122" s="17" t="n"/>
       <c r="C122" s="17" t="n"/>
@@ -1883,7 +1875,7 @@
       <c r="G122" s="18" t="n"/>
       <c r="H122" s="17" t="n"/>
     </row>
-    <row r="123">
+    <row r="123" ht="27" customHeight="1">
       <c r="A123" s="16" t="n"/>
       <c r="B123" s="17" t="n"/>
       <c r="C123" s="17" t="n"/>
@@ -1893,7 +1885,7 @@
       <c r="G123" s="18" t="n"/>
       <c r="H123" s="17" t="n"/>
     </row>
-    <row r="124">
+    <row r="124" ht="27" customHeight="1">
       <c r="A124" s="16" t="n"/>
       <c r="B124" s="17" t="n"/>
       <c r="C124" s="17" t="n"/>
@@ -1903,7 +1895,7 @@
       <c r="G124" s="18" t="n"/>
       <c r="H124" s="17" t="n"/>
     </row>
-    <row r="125">
+    <row r="125" ht="27" customHeight="1">
       <c r="A125" s="16" t="n"/>
       <c r="B125" s="17" t="n"/>
       <c r="C125" s="17" t="n"/>
@@ -1913,7 +1905,7 @@
       <c r="G125" s="18" t="n"/>
       <c r="H125" s="17" t="n"/>
     </row>
-    <row r="126">
+    <row r="126" ht="27" customHeight="1">
       <c r="A126" s="16" t="n"/>
       <c r="B126" s="17" t="n"/>
       <c r="C126" s="17" t="n"/>
@@ -1923,7 +1915,7 @@
       <c r="G126" s="18" t="n"/>
       <c r="H126" s="17" t="n"/>
     </row>
-    <row r="127">
+    <row r="127" ht="27" customHeight="1">
       <c r="A127" s="16" t="n"/>
       <c r="B127" s="17" t="n"/>
       <c r="C127" s="17" t="n"/>
@@ -1933,7 +1925,7 @@
       <c r="G127" s="18" t="n"/>
       <c r="H127" s="17" t="n"/>
     </row>
-    <row r="128">
+    <row r="128" ht="27" customHeight="1">
       <c r="A128" s="16" t="n"/>
       <c r="B128" s="17" t="n"/>
       <c r="C128" s="17" t="n"/>
@@ -1943,7 +1935,7 @@
       <c r="G128" s="18" t="n"/>
       <c r="H128" s="17" t="n"/>
     </row>
-    <row r="129">
+    <row r="129" ht="27" customHeight="1">
       <c r="A129" s="16" t="n"/>
       <c r="B129" s="17" t="n"/>
       <c r="C129" s="17" t="n"/>
@@ -1953,7 +1945,7 @@
       <c r="G129" s="18" t="n"/>
       <c r="H129" s="17" t="n"/>
     </row>
-    <row r="130">
+    <row r="130" ht="27" customHeight="1">
       <c r="A130" s="16" t="n"/>
       <c r="B130" s="17" t="n"/>
       <c r="C130" s="17" t="n"/>
@@ -1963,7 +1955,7 @@
       <c r="G130" s="18" t="n"/>
       <c r="H130" s="17" t="n"/>
     </row>
-    <row r="131">
+    <row r="131" ht="27" customHeight="1">
       <c r="A131" s="16" t="n"/>
       <c r="B131" s="17" t="n"/>
       <c r="C131" s="17" t="n"/>
@@ -1973,7 +1965,7 @@
       <c r="G131" s="18" t="n"/>
       <c r="H131" s="17" t="n"/>
     </row>
-    <row r="132">
+    <row r="132" ht="27" customHeight="1">
       <c r="A132" s="16" t="n"/>
       <c r="B132" s="17" t="n"/>
       <c r="C132" s="17" t="n"/>
@@ -1983,7 +1975,7 @@
       <c r="G132" s="18" t="n"/>
       <c r="H132" s="17" t="n"/>
     </row>
-    <row r="133">
+    <row r="133" ht="27" customHeight="1">
       <c r="A133" s="16" t="n"/>
       <c r="B133" s="17" t="n"/>
       <c r="C133" s="17" t="n"/>
@@ -1993,7 +1985,7 @@
       <c r="G133" s="18" t="n"/>
       <c r="H133" s="17" t="n"/>
     </row>
-    <row r="134">
+    <row r="134" ht="27" customHeight="1">
       <c r="A134" s="16" t="n"/>
       <c r="B134" s="17" t="n"/>
       <c r="C134" s="17" t="n"/>
@@ -2003,7 +1995,7 @@
       <c r="G134" s="18" t="n"/>
       <c r="H134" s="17" t="n"/>
     </row>
-    <row r="135">
+    <row r="135" ht="27" customHeight="1">
       <c r="A135" s="16" t="n"/>
       <c r="B135" s="17" t="n"/>
       <c r="C135" s="17" t="n"/>
@@ -2013,7 +2005,7 @@
       <c r="G135" s="18" t="n"/>
       <c r="H135" s="17" t="n"/>
     </row>
-    <row r="136">
+    <row r="136" ht="27" customHeight="1">
       <c r="A136" s="16" t="n"/>
       <c r="B136" s="17" t="n"/>
       <c r="C136" s="17" t="n"/>
@@ -2023,7 +2015,7 @@
       <c r="G136" s="18" t="n"/>
       <c r="H136" s="17" t="n"/>
     </row>
-    <row r="137">
+    <row r="137" ht="27" customHeight="1">
       <c r="A137" s="16" t="n"/>
       <c r="B137" s="17" t="n"/>
       <c r="C137" s="17" t="n"/>
@@ -2033,7 +2025,7 @@
       <c r="G137" s="18" t="n"/>
       <c r="H137" s="17" t="n"/>
     </row>
-    <row r="138">
+    <row r="138" ht="27" customHeight="1">
       <c r="A138" s="16" t="n"/>
       <c r="B138" s="17" t="n"/>
       <c r="C138" s="17" t="n"/>
@@ -2043,7 +2035,7 @@
       <c r="G138" s="18" t="n"/>
       <c r="H138" s="17" t="n"/>
     </row>
-    <row r="139">
+    <row r="139" ht="27" customHeight="1">
       <c r="A139" s="16" t="n"/>
       <c r="B139" s="17" t="n"/>
       <c r="C139" s="17" t="n"/>
@@ -2053,7 +2045,7 @@
       <c r="G139" s="18" t="n"/>
       <c r="H139" s="17" t="n"/>
     </row>
-    <row r="140">
+    <row r="140" ht="27" customHeight="1">
       <c r="A140" s="16" t="n"/>
       <c r="B140" s="17" t="n"/>
       <c r="C140" s="17" t="n"/>
@@ -2063,7 +2055,7 @@
       <c r="G140" s="18" t="n"/>
       <c r="H140" s="17" t="n"/>
     </row>
-    <row r="141">
+    <row r="141" ht="27" customHeight="1">
       <c r="A141" s="16" t="n"/>
       <c r="B141" s="17" t="n"/>
       <c r="C141" s="17" t="n"/>
@@ -2073,7 +2065,7 @@
       <c r="G141" s="18" t="n"/>
       <c r="H141" s="17" t="n"/>
     </row>
-    <row r="142">
+    <row r="142" ht="27" customHeight="1">
       <c r="A142" s="16" t="n"/>
       <c r="B142" s="17" t="n"/>
       <c r="C142" s="17" t="n"/>
@@ -2083,7 +2075,7 @@
       <c r="G142" s="18" t="n"/>
       <c r="H142" s="17" t="n"/>
     </row>
-    <row r="143">
+    <row r="143" ht="27" customHeight="1">
       <c r="A143" s="16" t="n"/>
       <c r="B143" s="17" t="n"/>
       <c r="C143" s="17" t="n"/>
@@ -2093,7 +2085,7 @@
       <c r="G143" s="18" t="n"/>
       <c r="H143" s="17" t="n"/>
     </row>
-    <row r="144">
+    <row r="144" ht="27" customHeight="1">
       <c r="A144" s="16" t="n"/>
       <c r="B144" s="17" t="n"/>
       <c r="C144" s="17" t="n"/>
@@ -2103,7 +2095,7 @@
       <c r="G144" s="18" t="n"/>
       <c r="H144" s="17" t="n"/>
     </row>
-    <row r="145">
+    <row r="145" ht="27" customHeight="1">
       <c r="A145" s="16" t="n"/>
       <c r="B145" s="17" t="n"/>
       <c r="C145" s="17" t="n"/>
@@ -2113,7 +2105,7 @@
       <c r="G145" s="18" t="n"/>
       <c r="H145" s="17" t="n"/>
     </row>
-    <row r="146">
+    <row r="146" ht="27" customHeight="1">
       <c r="A146" s="16" t="n"/>
       <c r="B146" s="17" t="n"/>
       <c r="C146" s="17" t="n"/>
@@ -2123,7 +2115,7 @@
       <c r="G146" s="18" t="n"/>
       <c r="H146" s="17" t="n"/>
     </row>
-    <row r="147">
+    <row r="147" ht="27" customHeight="1">
       <c r="A147" s="16" t="n"/>
       <c r="B147" s="17" t="n"/>
       <c r="C147" s="17" t="n"/>
@@ -2133,7 +2125,7 @@
       <c r="G147" s="18" t="n"/>
       <c r="H147" s="17" t="n"/>
     </row>
-    <row r="148">
+    <row r="148" ht="27" customHeight="1">
       <c r="A148" s="16" t="n"/>
       <c r="B148" s="17" t="n"/>
       <c r="C148" s="17" t="n"/>
@@ -2143,7 +2135,7 @@
       <c r="G148" s="18" t="n"/>
       <c r="H148" s="17" t="n"/>
     </row>
-    <row r="149">
+    <row r="149" ht="27" customHeight="1">
       <c r="A149" s="16" t="n"/>
       <c r="B149" s="17" t="n"/>
       <c r="C149" s="17" t="n"/>
@@ -2153,7 +2145,7 @@
       <c r="G149" s="18" t="n"/>
       <c r="H149" s="17" t="n"/>
     </row>
-    <row r="150">
+    <row r="150" ht="27" customHeight="1">
       <c r="A150" s="16" t="n"/>
       <c r="B150" s="17" t="n"/>
       <c r="C150" s="17" t="n"/>
@@ -2163,7 +2155,7 @@
       <c r="G150" s="18" t="n"/>
       <c r="H150" s="17" t="n"/>
     </row>
-    <row r="151">
+    <row r="151" ht="27" customHeight="1">
       <c r="A151" s="16" t="n"/>
       <c r="B151" s="17" t="n"/>
       <c r="C151" s="17" t="n"/>
@@ -2173,7 +2165,7 @@
       <c r="G151" s="18" t="n"/>
       <c r="H151" s="17" t="n"/>
     </row>
-    <row r="152">
+    <row r="152" ht="27" customHeight="1">
       <c r="A152" s="16" t="n"/>
       <c r="B152" s="17" t="n"/>
       <c r="C152" s="17" t="n"/>
@@ -2183,7 +2175,7 @@
       <c r="G152" s="18" t="n"/>
       <c r="H152" s="17" t="n"/>
     </row>
-    <row r="153">
+    <row r="153" ht="27" customHeight="1">
       <c r="A153" s="16" t="n"/>
       <c r="B153" s="17" t="n"/>
       <c r="C153" s="17" t="n"/>
@@ -2193,7 +2185,7 @@
       <c r="G153" s="18" t="n"/>
       <c r="H153" s="17" t="n"/>
     </row>
-    <row r="154">
+    <row r="154" ht="27" customHeight="1">
       <c r="A154" s="16" t="n"/>
       <c r="B154" s="17" t="n"/>
       <c r="C154" s="17" t="n"/>
@@ -2203,7 +2195,7 @@
       <c r="G154" s="18" t="n"/>
       <c r="H154" s="17" t="n"/>
     </row>
-    <row r="155">
+    <row r="155" ht="27" customHeight="1">
       <c r="A155" s="16" t="n"/>
       <c r="B155" s="17" t="n"/>
       <c r="C155" s="17" t="n"/>
@@ -2213,7 +2205,7 @@
       <c r="G155" s="18" t="n"/>
       <c r="H155" s="17" t="n"/>
     </row>
-    <row r="156">
+    <row r="156" ht="27" customHeight="1">
       <c r="A156" s="16" t="n"/>
       <c r="B156" s="17" t="n"/>
       <c r="C156" s="17" t="n"/>
@@ -2223,7 +2215,7 @@
       <c r="G156" s="18" t="n"/>
       <c r="H156" s="17" t="n"/>
     </row>
-    <row r="157">
+    <row r="157" ht="27" customHeight="1">
       <c r="A157" s="16" t="n"/>
       <c r="B157" s="17" t="n"/>
       <c r="C157" s="17" t="n"/>
@@ -2233,7 +2225,7 @@
       <c r="G157" s="18" t="n"/>
       <c r="H157" s="17" t="n"/>
     </row>
-    <row r="158">
+    <row r="158" ht="27" customHeight="1">
       <c r="A158" s="16" t="n"/>
       <c r="B158" s="17" t="n"/>
       <c r="C158" s="17" t="n"/>
@@ -2243,7 +2235,7 @@
       <c r="G158" s="18" t="n"/>
       <c r="H158" s="17" t="n"/>
     </row>
-    <row r="159">
+    <row r="159" ht="27" customHeight="1">
       <c r="A159" s="16" t="n"/>
       <c r="B159" s="17" t="n"/>
       <c r="C159" s="17" t="n"/>
@@ -2253,7 +2245,7 @@
       <c r="G159" s="18" t="n"/>
       <c r="H159" s="17" t="n"/>
     </row>
-    <row r="160">
+    <row r="160" ht="27" customHeight="1">
       <c r="A160" s="16" t="n"/>
       <c r="B160" s="17" t="n"/>
       <c r="C160" s="17" t="n"/>
@@ -2263,7 +2255,7 @@
       <c r="G160" s="18" t="n"/>
       <c r="H160" s="17" t="n"/>
     </row>
-    <row r="161">
+    <row r="161" ht="27" customHeight="1">
       <c r="A161" s="16" t="n"/>
       <c r="B161" s="17" t="n"/>
       <c r="C161" s="17" t="n"/>
@@ -2273,7 +2265,7 @@
       <c r="G161" s="18" t="n"/>
       <c r="H161" s="17" t="n"/>
     </row>
-    <row r="162">
+    <row r="162" ht="27" customHeight="1">
       <c r="A162" s="16" t="n"/>
       <c r="B162" s="17" t="n"/>
       <c r="C162" s="17" t="n"/>
@@ -2283,7 +2275,7 @@
       <c r="G162" s="18" t="n"/>
       <c r="H162" s="17" t="n"/>
     </row>
-    <row r="163">
+    <row r="163" ht="27" customHeight="1">
       <c r="A163" s="16" t="n"/>
       <c r="B163" s="17" t="n"/>
       <c r="C163" s="17" t="n"/>
@@ -2293,7 +2285,7 @@
       <c r="G163" s="18" t="n"/>
       <c r="H163" s="17" t="n"/>
     </row>
-    <row r="164">
+    <row r="164" ht="27" customHeight="1">
       <c r="A164" s="16" t="n"/>
       <c r="B164" s="17" t="n"/>
       <c r="C164" s="17" t="n"/>
@@ -2303,7 +2295,7 @@
       <c r="G164" s="18" t="n"/>
       <c r="H164" s="17" t="n"/>
     </row>
-    <row r="165">
+    <row r="165" ht="27" customHeight="1">
       <c r="A165" s="16" t="n"/>
       <c r="B165" s="17" t="n"/>
       <c r="C165" s="17" t="n"/>
@@ -2313,7 +2305,7 @@
       <c r="G165" s="18" t="n"/>
       <c r="H165" s="17" t="n"/>
     </row>
-    <row r="166">
+    <row r="166" ht="27" customHeight="1">
       <c r="A166" s="16" t="n"/>
       <c r="B166" s="17" t="n"/>
       <c r="C166" s="17" t="n"/>
@@ -2323,7 +2315,7 @@
       <c r="G166" s="18" t="n"/>
       <c r="H166" s="17" t="n"/>
     </row>
-    <row r="167">
+    <row r="167" ht="27" customHeight="1">
       <c r="A167" s="16" t="n"/>
       <c r="B167" s="17" t="n"/>
       <c r="C167" s="17" t="n"/>
@@ -2333,7 +2325,7 @@
       <c r="G167" s="18" t="n"/>
       <c r="H167" s="17" t="n"/>
     </row>
-    <row r="168">
+    <row r="168" ht="27" customHeight="1">
       <c r="A168" s="16" t="n"/>
       <c r="B168" s="17" t="n"/>
       <c r="C168" s="17" t="n"/>
@@ -2343,7 +2335,7 @@
       <c r="G168" s="18" t="n"/>
       <c r="H168" s="17" t="n"/>
     </row>
-    <row r="169">
+    <row r="169" ht="27" customHeight="1">
       <c r="A169" s="16" t="n"/>
       <c r="B169" s="17" t="n"/>
       <c r="C169" s="17" t="n"/>
@@ -2353,7 +2345,7 @@
       <c r="G169" s="18" t="n"/>
       <c r="H169" s="17" t="n"/>
     </row>
-    <row r="170">
+    <row r="170" ht="27" customHeight="1">
       <c r="A170" s="16" t="n"/>
       <c r="B170" s="17" t="n"/>
       <c r="C170" s="17" t="n"/>
@@ -2363,7 +2355,7 @@
       <c r="G170" s="18" t="n"/>
       <c r="H170" s="17" t="n"/>
     </row>
-    <row r="171">
+    <row r="171" ht="27" customHeight="1">
       <c r="A171" s="19" t="n"/>
       <c r="B171" s="20" t="n"/>
       <c r="C171" s="20" t="n"/>
@@ -2373,45 +2365,45 @@
       <c r="G171" s="21" t="n"/>
       <c r="H171" s="20" t="n"/>
     </row>
-    <row r="173" ht="19" customHeight="1">
+    <row r="173" ht="17" customHeight="1">
       <c r="E173" s="22" t="inlineStr">
         <is>
           <t>小　　計</t>
         </is>
       </c>
-      <c r="G173" s="18" t="n"/>
-    </row>
-    <row r="174" ht="19" customHeight="1">
+      <c r="G173" s="23" t="n"/>
+    </row>
+    <row r="174" ht="17" customHeight="1">
       <c r="E174" s="22" t="inlineStr">
         <is>
           <t>値 引 き</t>
         </is>
       </c>
-      <c r="G174" s="18" t="n"/>
-    </row>
-    <row r="175" ht="19" customHeight="1">
+      <c r="G174" s="23" t="n"/>
+    </row>
+    <row r="175" ht="17" customHeight="1">
       <c r="E175" s="22" t="inlineStr">
         <is>
           <t>税抜合計</t>
         </is>
       </c>
-      <c r="G175" s="18" t="n"/>
-    </row>
-    <row r="176" ht="19" customHeight="1">
+      <c r="G175" s="23" t="n"/>
+    </row>
+    <row r="176" ht="17" customHeight="1">
       <c r="E176" s="22" t="inlineStr">
         <is>
           <t>消 費 税</t>
         </is>
       </c>
-      <c r="G176" s="18" t="n"/>
-    </row>
-    <row r="177" ht="26" customHeight="1">
-      <c r="E177" s="23" t="inlineStr">
+      <c r="G176" s="23" t="n"/>
+    </row>
+    <row r="177" ht="23" customHeight="1">
+      <c r="E177" s="24" t="inlineStr">
         <is>
           <t>税込合計</t>
         </is>
       </c>
-      <c r="G177" s="24" t="n"/>
+      <c r="G177" s="25" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="5" t="inlineStr">
@@ -2419,12 +2411,12 @@
           <t>備考</t>
         </is>
       </c>
-      <c r="B179" s="25" t="n"/>
+      <c r="B179" s="26" t="n"/>
     </row>
     <row r="180"/>
     <row r="181"/>
     <row r="183">
-      <c r="A183" s="26" t="inlineStr">
+      <c r="A183" s="27" t="inlineStr">
         <is>
           <t>※本見積書の有効期限を過ぎた場合は、再度お見積りいたします。</t>
         </is>

</xml_diff>

<commit_message>
Repeat the item header as real cells on continuation pages
Numbers ignores Excel's print-title-rows setting, so the second page of a
long quote arrived with no column header even though LibreOffice rendered
it correctly. Stop relying on a print setting: write the header row into
the sheet at each page boundary and add an explicit page break there, so
the repeat survives in any application.

- emit the header row as data every FIRST/NEXT_PAGE_ITEM_ROWS lines and
  drop print_title_rows, which would otherwise double up
- trim header and totals/remark spacing, and shorten the remark box to
  two rows, so an ordinary estimate still fits one sheet
- only fit-to-height when no break was inserted

Verified 3, 6, 16, 19 and 40 line estimates paginate as 1/1/1/2/4 quote
pages, each continuation page carrying the header.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/test_cyca_estimate_single_sheet_template.xlsx
+++ b/templates/test_cyca_estimate_single_sheet_template.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積書" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'見積書'!$A$1:$H$183</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'見積書'!$A$1:$H$182</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H183"/>
+  <dimension ref="A2:H182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -697,6 +697,7 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="8" customHeight="1"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -724,6 +725,7 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -733,7 +735,7 @@
       <c r="C10" s="8" t="n"/>
     </row>
     <row r="11" ht="17" customHeight="1"/>
-    <row r="12">
+    <row r="12" ht="12" customHeight="1">
       <c r="C12" s="9" t="inlineStr">
         <is>
           <t>（消費税込）</t>
@@ -816,6 +818,7 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="8" customHeight="1"/>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
@@ -2365,6 +2368,7 @@
       <c r="G171" s="21" t="n"/>
       <c r="H171" s="20" t="n"/>
     </row>
+    <row r="172" ht="6" customHeight="1"/>
     <row r="173" ht="17" customHeight="1">
       <c r="E173" s="22" t="inlineStr">
         <is>
@@ -2405,6 +2409,7 @@
       </c>
       <c r="G177" s="25" t="n"/>
     </row>
+    <row r="178" ht="6" customHeight="1"/>
     <row r="179">
       <c r="A179" s="5" t="inlineStr">
         <is>
@@ -2414,9 +2419,9 @@
       <c r="B179" s="26" t="n"/>
     </row>
     <row r="180"/>
-    <row r="181"/>
-    <row r="183">
-      <c r="A183" s="27" t="inlineStr">
+    <row r="181" ht="6" customHeight="1"/>
+    <row r="182" ht="12" customHeight="1">
+      <c r="A182" s="27" t="inlineStr">
         <is>
           <t>※本見積書の有効期限を過ぎた場合は、再度お見積りいたします。</t>
         </is>
@@ -2427,14 +2432,15 @@
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="E175:F175"/>
+    <mergeCell ref="A182:H182"/>
     <mergeCell ref="E16:H16"/>
     <mergeCell ref="C14:D14"/>
+    <mergeCell ref="B179:H180"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="G7:H7"/>
-    <mergeCell ref="A183:H183"/>
     <mergeCell ref="E177:F177"/>
     <mergeCell ref="A10:B11"/>
     <mergeCell ref="A18:B18"/>
@@ -2450,7 +2456,6 @@
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="E13:H13"/>
     <mergeCell ref="A20:H20"/>
-    <mergeCell ref="B179:H181"/>
     <mergeCell ref="E174:F174"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="E15:H15"/>

</xml_diff>

<commit_message>
Pin the print scale so page breaks land where intended
The repeated header still missed the top of page two in Numbers. Numbers
has no manual page breaks and ignores the ones written into the file, and
with fit-to-width each application picked its own scale, so the header
row written into the sheet sat wherever that application happened to
break rather than at the boundary.

Fix the scale at 85% instead of fitting to width, so every application
paginates identically, and measure the real capacity at that scale:
21 item rows on page one, 15 when the totals share the page, 24 on later
pages. _plan_pages() distributes rows against those numbers and keeps the
last page wide enough for the totals, so they are never stranded alone.

Verified at 10/15/16/19/20/21/25/30/38/45/60 rows: every continuation page
opens with the header and no page holds only the totals.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/test_cyca_estimate_single_sheet_template.xlsx
+++ b/templates/test_cyca_estimate_single_sheet_template.xlsx
@@ -665,7 +665,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A2:H182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2463,7 +2463,7 @@
     <mergeCell ref="C18:D18"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="85"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>